<commit_message>
@ Added task history system and Excel-based input support @ Implemented task history tracking and load tasks from Excel file @ Added history logs, task state tracking and Excel import support
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fardi\ByteForge\Task_Scheduler_Simulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5B416FF-02ED-4F04-8B53-877B9AAD8679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4985BD0F-3436-49E0-96A9-809EEA0DC372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{05F6162E-13F5-43DD-9C92-5B9D6672AF89}"/>
   </bookViews>
@@ -466,93 +466,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DFCA6AF-A4C3-482A-A34B-9EE9B1C13060}">
-  <dimension ref="I9:M13"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" width="2.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="9:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I9" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="9:13" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I10" s="2" t="s">
+    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J10" s="2">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="K10" s="2">
+      <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="L10" s="2">
+      <c r="D2" s="2">
         <v>3</v>
       </c>
-      <c r="M10" s="2"/>
+      <c r="E2" s="2"/>
     </row>
-    <row r="11" spans="9:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="I11" s="2" t="s">
+    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="B3" s="2">
         <v>3</v>
       </c>
-      <c r="K11" s="2">
+      <c r="C3" s="2">
         <v>2</v>
       </c>
-      <c r="L11" s="2">
+      <c r="D3" s="2">
         <v>-1</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="9:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="I12" s="2" t="s">
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J12" s="2">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="K12" s="2">
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="L12" s="2">
+      <c r="D4" s="2">
         <v>-1</v>
       </c>
-      <c r="M12" s="2"/>
+      <c r="E4" s="2"/>
     </row>
-    <row r="13" spans="9:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="I13" s="2" t="s">
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J13" s="2">
+      <c r="B5" s="2">
         <v>3</v>
       </c>
-      <c r="K13" s="2">
+      <c r="C5" s="2">
         <v>1</v>
       </c>
-      <c r="L13" s="2">
+      <c r="D5" s="2">
         <v>-1</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="9" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:5" ht="46.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
@ feat: add task history and Excel-driven simulation @ Add task history and Excel input support @ Your branch is behind 'origin/master' by 1 commit
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fardi\ByteForge\Task_Scheduler_Simulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4985BD0F-3436-49E0-96A9-809EEA0DC372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469AF93A-DA6F-4B8E-AEF7-53E6B7F1792D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{05F6162E-13F5-43DD-9C92-5B9D6672AF89}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="9960" xr2:uid="{05F6162E-13F5-43DD-9C92-5B9D6672AF89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>